<commit_message>
chore: actualiza resultados de estimación, métricas e imágenes
</commit_message>
<xml_diff>
--- a/data/processed/df_rec_peso_pnd25.xlsx
+++ b/data/processed/df_rec_peso_pnd25.xlsx
@@ -1064,7 +1064,7 @@
         <v>23.5</v>
       </c>
       <c r="E37" t="n">
-        <v>1.007636707833906</v>
+        <v>1.007636707833905</v>
       </c>
     </row>
     <row r="38">
@@ -1506,7 +1506,7 @@
         <v>22.8</v>
       </c>
       <c r="E63" t="n">
-        <v>0.9033006222888622</v>
+        <v>0.9033006222888621</v>
       </c>
     </row>
     <row r="64">
@@ -1523,7 +1523,7 @@
         <v>13.3</v>
       </c>
       <c r="E64" t="n">
-        <v>-0.7266058109575452</v>
+        <v>-0.726605810957545</v>
       </c>
     </row>
     <row r="65">
@@ -1540,7 +1540,7 @@
         <v>13.1</v>
       </c>
       <c r="E65" t="n">
-        <v>-0.758004233319085</v>
+        <v>-0.7580042333190848</v>
       </c>
     </row>
     <row r="66">
@@ -1557,7 +1557,7 @@
         <v>11</v>
       </c>
       <c r="E66" t="n">
-        <v>-1.385697781068808</v>
+        <v>-1.385697781068807</v>
       </c>
     </row>
     <row r="67">
@@ -1676,7 +1676,7 @@
         <v>22.2</v>
       </c>
       <c r="E73" t="n">
-        <v>0.8161498870226594</v>
+        <v>0.8161498870226596</v>
       </c>
     </row>
     <row r="74">
@@ -1727,7 +1727,7 @@
         <v>13.3</v>
       </c>
       <c r="E76" t="n">
-        <v>-0.7266058109575452</v>
+        <v>-0.726605810957545</v>
       </c>
     </row>
     <row r="77">
@@ -1744,7 +1744,7 @@
         <v>26.72</v>
       </c>
       <c r="E77" t="n">
-        <v>1.329601910801645</v>
+        <v>1.329601910801646</v>
       </c>
     </row>
     <row r="78">
@@ -1829,7 +1829,7 @@
         <v>25.96</v>
       </c>
       <c r="E82" t="n">
-        <v>1.253004046434014</v>
+        <v>1.253004046434013</v>
       </c>
     </row>
     <row r="83">
@@ -1880,7 +1880,7 @@
         <v>23.35</v>
       </c>
       <c r="E85" t="n">
-        <v>0.9903269827862897</v>
+        <v>0.9903269827862901</v>
       </c>
     </row>
     <row r="86">
@@ -2543,7 +2543,7 @@
         <v>11.21</v>
       </c>
       <c r="E124" t="n">
-        <v>-1.275302474602154</v>
+        <v>-1.275302474602153</v>
       </c>
     </row>
     <row r="125">
@@ -2611,7 +2611,7 @@
         <v>22.89</v>
       </c>
       <c r="E128" t="n">
-        <v>0.9108728690353499</v>
+        <v>0.91087286903535</v>
       </c>
     </row>
     <row r="129">
@@ -2747,7 +2747,7 @@
         <v>23.25</v>
       </c>
       <c r="E136" t="n">
-        <v>0.9742420296454317</v>
+        <v>0.9742420296454318</v>
       </c>
     </row>
     <row r="137">
@@ -2832,7 +2832,7 @@
         <v>22.42</v>
       </c>
       <c r="E141" t="n">
-        <v>0.8519733284846679</v>
+        <v>0.851973328484668</v>
       </c>
     </row>
     <row r="142">
@@ -3240,7 +3240,7 @@
         <v>23.11</v>
       </c>
       <c r="E165" t="n">
-        <v>0.9575645400304821</v>
+        <v>0.9575645400304822</v>
       </c>
     </row>
     <row r="166">
@@ -4362,7 +4362,7 @@
         <v>22.89</v>
       </c>
       <c r="E231" t="n">
-        <v>0.9108728690353499</v>
+        <v>0.91087286903535</v>
       </c>
     </row>
     <row r="232">
@@ -4787,7 +4787,7 @@
         <v>12.12</v>
       </c>
       <c r="E256" t="n">
-        <v>-1.035789621854488</v>
+        <v>-1.035789621854487</v>
       </c>
     </row>
     <row r="257">
@@ -5331,7 +5331,7 @@
         <v>13.3</v>
       </c>
       <c r="E288" t="n">
-        <v>-0.7266058109575452</v>
+        <v>-0.726605810957545</v>
       </c>
     </row>
     <row r="289">
@@ -5382,7 +5382,7 @@
         <v>22.8</v>
       </c>
       <c r="E291" t="n">
-        <v>0.9033006222888622</v>
+        <v>0.9033006222888621</v>
       </c>
     </row>
     <row r="292">
@@ -5433,7 +5433,7 @@
         <v>13.1</v>
       </c>
       <c r="E294" t="n">
-        <v>-0.758004233319085</v>
+        <v>-0.7580042333190848</v>
       </c>
     </row>
     <row r="295">
@@ -5620,7 +5620,7 @@
         <v>21.8</v>
       </c>
       <c r="E305" t="n">
-        <v>0.7546642694731029</v>
+        <v>0.7546642694731031</v>
       </c>
     </row>
     <row r="306">
@@ -5654,7 +5654,7 @@
         <v>22.2</v>
       </c>
       <c r="E307" t="n">
-        <v>0.8161498870226594</v>
+        <v>0.8161498870226596</v>
       </c>
     </row>
     <row r="308">
@@ -5858,7 +5858,7 @@
         <v>12.3</v>
       </c>
       <c r="E319" t="n">
-        <v>-0.9979196589738004</v>
+        <v>-0.9979196589738006</v>
       </c>
     </row>
     <row r="320">
@@ -6079,7 +6079,7 @@
         <v>22.2</v>
       </c>
       <c r="E332" t="n">
-        <v>0.8161498870226594</v>
+        <v>0.8161498870226596</v>
       </c>
     </row>
     <row r="333">
@@ -6351,7 +6351,7 @@
         <v>23.3</v>
       </c>
       <c r="E348" t="n">
-        <v>0.9839844620698338</v>
+        <v>0.9839844620698337</v>
       </c>
     </row>
     <row r="349">
@@ -6759,7 +6759,7 @@
         <v>23.44</v>
       </c>
       <c r="E372" t="n">
-        <v>0.9973163154080958</v>
+        <v>0.9973163154080956</v>
       </c>
     </row>
     <row r="373">
@@ -6827,7 +6827,7 @@
         <v>23.27</v>
       </c>
       <c r="E376" t="n">
-        <v>0.9773375885524462</v>
+        <v>0.977337588552446</v>
       </c>
     </row>
     <row r="377">
@@ -7082,7 +7082,7 @@
         <v>22.39</v>
       </c>
       <c r="E391" t="n">
-        <v>0.8463227100467087</v>
+        <v>0.8463227100467086</v>
       </c>
     </row>
     <row r="392">
@@ -7218,7 +7218,7 @@
         <v>59.66</v>
       </c>
       <c r="E399" t="n">
-        <v>3.287437061543074</v>
+        <v>3.287437061543073</v>
       </c>
     </row>
     <row r="400">
@@ -7643,7 +7643,7 @@
         <v>22.2</v>
       </c>
       <c r="E424" t="n">
-        <v>0.8161498870226594</v>
+        <v>0.8161498870226596</v>
       </c>
     </row>
     <row r="425">
@@ -7813,7 +7813,7 @@
         <v>32.53</v>
       </c>
       <c r="E434" t="n">
-        <v>1.797036925001075</v>
+        <v>1.797036925001074</v>
       </c>
     </row>
     <row r="435">
@@ -7915,7 +7915,7 @@
         <v>22.69</v>
       </c>
       <c r="E440" t="n">
-        <v>0.8883093448377877</v>
+        <v>0.8883093448377878</v>
       </c>
     </row>
     <row r="441">
@@ -7966,7 +7966,7 @@
         <v>30.74</v>
       </c>
       <c r="E443" t="n">
-        <v>1.694442626838635</v>
+        <v>1.694442626838634</v>
       </c>
     </row>
     <row r="444">
@@ -8051,7 +8051,7 @@
         <v>30.19</v>
       </c>
       <c r="E448" t="n">
-        <v>1.651319838353589</v>
+        <v>1.65131983835359</v>
       </c>
     </row>
     <row r="449">
@@ -8459,7 +8459,7 @@
         <v>20.05</v>
       </c>
       <c r="E472" t="n">
-        <v>0.5487650819475514</v>
+        <v>0.5487650819475512</v>
       </c>
     </row>
     <row r="473">
@@ -8476,7 +8476,7 @@
         <v>30.04</v>
       </c>
       <c r="E473" t="n">
-        <v>1.628611346296881</v>
+        <v>1.62861134629688</v>
       </c>
     </row>
     <row r="474">
@@ -9360,7 +9360,7 @@
         <v>11.21</v>
       </c>
       <c r="E525" t="n">
-        <v>-1.275302474602154</v>
+        <v>-1.275302474602153</v>
       </c>
     </row>
     <row r="526">
@@ -9530,7 +9530,7 @@
         <v>34.33</v>
       </c>
       <c r="E535" t="n">
-        <v>1.91253536164872</v>
+        <v>1.912535361648721</v>
       </c>
     </row>
     <row r="536">
@@ -10040,7 +10040,7 @@
         <v>34.89</v>
       </c>
       <c r="E565" t="n">
-        <v>1.947475877816469</v>
+        <v>1.947475877816468</v>
       </c>
     </row>
     <row r="566">
@@ -10142,7 +10142,7 @@
         <v>22.06</v>
       </c>
       <c r="E571" t="n">
-        <v>0.7860204598235619</v>
+        <v>0.7860204598235621</v>
       </c>
     </row>
     <row r="572">
@@ -10244,7 +10244,7 @@
         <v>25.73</v>
       </c>
       <c r="E577" t="n">
-        <v>1.229297311621018</v>
+        <v>1.229297311621017</v>
       </c>
     </row>
     <row r="578">
@@ -10788,7 +10788,7 @@
         <v>12.44</v>
       </c>
       <c r="E609" t="n">
-        <v>-0.9539797406561978</v>
+        <v>-0.9539797406561981</v>
       </c>
     </row>
     <row r="610">
@@ -11553,7 +11553,7 @@
         <v>7.92</v>
       </c>
       <c r="E654" t="n">
-        <v>-2.345629180282807</v>
+        <v>-2.345629180282806</v>
       </c>
     </row>
     <row r="655">
@@ -11604,7 +11604,7 @@
         <v>9.31</v>
       </c>
       <c r="E657" t="n">
-        <v>-1.9471710165722</v>
+        <v>-1.947171016572199</v>
       </c>
     </row>
     <row r="658">
@@ -11655,7 +11655,7 @@
         <v>11.62</v>
       </c>
       <c r="E660" t="n">
-        <v>-1.18866565213657</v>
+        <v>-1.188665652136569</v>
       </c>
     </row>
     <row r="661">
@@ -12199,7 +12199,7 @@
         <v>13.1</v>
       </c>
       <c r="E692" t="n">
-        <v>-0.758004233319085</v>
+        <v>-0.7580042333190848</v>
       </c>
     </row>
     <row r="693">
@@ -12301,7 +12301,7 @@
         <v>23.01</v>
       </c>
       <c r="E698" t="n">
-        <v>0.9393188190188101</v>
+        <v>0.93931881901881</v>
       </c>
     </row>
     <row r="699">
@@ -12488,7 +12488,7 @@
         <v>12.15</v>
       </c>
       <c r="E709" t="n">
-        <v>-1.021408889666503</v>
+        <v>-1.021408889666502</v>
       </c>
     </row>
     <row r="710">
@@ -12539,7 +12539,7 @@
         <v>22.21</v>
       </c>
       <c r="E712" t="n">
-        <v>0.8229721372811597</v>
+        <v>0.8229721372811596</v>
       </c>
     </row>
     <row r="713">
@@ -12675,7 +12675,7 @@
         <v>23.21</v>
       </c>
       <c r="E720" t="n">
-        <v>0.9649991407397237</v>
+        <v>0.9649991407397238</v>
       </c>
     </row>
     <row r="721">
@@ -13049,7 +13049,7 @@
         <v>23.86</v>
       </c>
       <c r="E742" t="n">
-        <v>1.049379491170712</v>
+        <v>1.049379491170711</v>
       </c>
     </row>
     <row r="743">
@@ -13270,7 +13270,7 @@
         <v>23.01</v>
       </c>
       <c r="E755" t="n">
-        <v>0.9393188190188101</v>
+        <v>0.93931881901881</v>
       </c>
     </row>
     <row r="756">
@@ -13355,7 +13355,7 @@
         <v>12.37</v>
       </c>
       <c r="E760" t="n">
-        <v>-0.9856104168672697</v>
+        <v>-0.9856104168672699</v>
       </c>
     </row>
     <row r="761">
@@ -13695,7 +13695,7 @@
         <v>12.49</v>
       </c>
       <c r="E780" t="n">
-        <v>-0.9339099412610544</v>
+        <v>-0.9339099412610545</v>
       </c>
     </row>
     <row r="781">
@@ -13746,7 +13746,7 @@
         <v>12.49</v>
       </c>
       <c r="E783" t="n">
-        <v>-0.9339099412610544</v>
+        <v>-0.9339099412610545</v>
       </c>
     </row>
     <row r="784">
@@ -13797,7 +13797,7 @@
         <v>34.46</v>
       </c>
       <c r="E786" t="n">
-        <v>1.924846792355398</v>
+        <v>1.924846792355399</v>
       </c>
     </row>
     <row r="787">
@@ -14052,7 +14052,7 @@
         <v>28.5</v>
       </c>
       <c r="E801" t="n">
-        <v>1.497843624110341</v>
+        <v>1.49784362411034</v>
       </c>
     </row>
     <row r="802">
@@ -14205,7 +14205,7 @@
         <v>12.37</v>
       </c>
       <c r="E810" t="n">
-        <v>-0.9856104168672697</v>
+        <v>-0.9856104168672699</v>
       </c>
     </row>
     <row r="811">
@@ -14902,7 +14902,7 @@
         <v>21.64</v>
       </c>
       <c r="E851" t="n">
-        <v>0.7418625517725864</v>
+        <v>0.7418625517725865</v>
       </c>
     </row>
     <row r="852">
@@ -15021,7 +15021,7 @@
         <v>23.05</v>
       </c>
       <c r="E858" t="n">
-        <v>0.9505292832151184</v>
+        <v>0.9505292832151185</v>
       </c>
     </row>
     <row r="859">
@@ -15106,7 +15106,7 @@
         <v>23.31</v>
       </c>
       <c r="E863" t="n">
-        <v>0.9862383071886068</v>
+        <v>0.9862383071886067</v>
       </c>
     </row>
     <row r="864">
@@ -15429,7 +15429,7 @@
         <v>22.69</v>
       </c>
       <c r="E882" t="n">
-        <v>0.8883093448377877</v>
+        <v>0.8883093448377878</v>
       </c>
     </row>
     <row r="883">
@@ -15718,7 +15718,7 @@
         <v>11.01</v>
       </c>
       <c r="E899" t="n">
-        <v>-1.380321478262939</v>
+        <v>-1.38032147826294</v>
       </c>
     </row>
     <row r="900">
@@ -15939,7 +15939,7 @@
         <v>25.48</v>
       </c>
       <c r="E912" t="n">
-        <v>1.204916615613179</v>
+        <v>1.204916615613178</v>
       </c>
     </row>
     <row r="913">
@@ -16619,7 +16619,7 @@
         <v>21.8</v>
       </c>
       <c r="E952" t="n">
-        <v>0.7546642694731029</v>
+        <v>0.7546642694731031</v>
       </c>
     </row>
     <row r="953">
@@ -16653,7 +16653,7 @@
         <v>11.94</v>
       </c>
       <c r="E954" t="n">
-        <v>-1.100909698511587</v>
+        <v>-1.100909698511586</v>
       </c>
     </row>
     <row r="955">
@@ -16874,7 +16874,7 @@
         <v>11.29</v>
       </c>
       <c r="E967" t="n">
-        <v>-1.256459886564349</v>
+        <v>-1.256459886564348</v>
       </c>
     </row>
     <row r="968">
@@ -17333,7 +17333,7 @@
         <v>18.69</v>
       </c>
       <c r="E994" t="n">
-        <v>0.3137715137338839</v>
+        <v>0.3137715137338838</v>
       </c>
     </row>
     <row r="995">
@@ -17775,7 +17775,7 @@
         <v>12.37</v>
       </c>
       <c r="E1020" t="n">
-        <v>-0.9856104168672697</v>
+        <v>-0.9856104168672699</v>
       </c>
     </row>
     <row r="1021">
@@ -19016,7 +19016,7 @@
         <v>11.02</v>
       </c>
       <c r="E1093" t="n">
-        <v>-1.371657225572654</v>
+        <v>-1.371657225572653</v>
       </c>
     </row>
     <row r="1094">
@@ -19084,7 +19084,7 @@
         <v>11.34</v>
       </c>
       <c r="E1097" t="n">
-        <v>-1.248263713316413</v>
+        <v>-1.248263713316412</v>
       </c>
     </row>
     <row r="1098">
@@ -19594,7 +19594,7 @@
         <v>12.37</v>
       </c>
       <c r="E1127" t="n">
-        <v>-0.9856104168672697</v>
+        <v>-0.9856104168672699</v>
       </c>
     </row>
     <row r="1128">
@@ -20206,7 +20206,7 @@
         <v>12.12</v>
       </c>
       <c r="E1163" t="n">
-        <v>-1.035789621854488</v>
+        <v>-1.035789621854487</v>
       </c>
     </row>
     <row r="1164">
@@ -20376,7 +20376,7 @@
         <v>22.46</v>
       </c>
       <c r="E1173" t="n">
-        <v>0.8551807022943996</v>
+        <v>0.8551807022943995</v>
       </c>
     </row>
     <row r="1174">
@@ -20461,7 +20461,7 @@
         <v>12.3</v>
       </c>
       <c r="E1178" t="n">
-        <v>-0.9979196589738004</v>
+        <v>-0.9979196589738006</v>
       </c>
     </row>
     <row r="1179">
@@ -20580,7 +20580,7 @@
         <v>12.52</v>
       </c>
       <c r="E1185" t="n">
-        <v>-0.9230023012010868</v>
+        <v>-0.9230023012010867</v>
       </c>
     </row>
     <row r="1186">
@@ -20835,7 +20835,7 @@
         <v>12.52</v>
       </c>
       <c r="E1200" t="n">
-        <v>-0.9230023012010868</v>
+        <v>-0.9230023012010867</v>
       </c>
     </row>
     <row r="1201">
@@ -21039,7 +21039,7 @@
         <v>11.02</v>
       </c>
       <c r="E1212" t="n">
-        <v>-1.371657225572654</v>
+        <v>-1.371657225572653</v>
       </c>
     </row>
     <row r="1213">
@@ -21124,7 +21124,7 @@
         <v>12.31</v>
       </c>
       <c r="E1217" t="n">
-        <v>-0.9950774840601946</v>
+        <v>-0.9950774840601945</v>
       </c>
     </row>
     <row r="1218">

</xml_diff>